<commit_message>
Update example/test files, add schedule generator and guide
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test/block 10 data.xlsx
+++ b/Test/block 10 data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/colin/Library/Mobile Documents/com~apple~CloudDocs/cbproj/scheduling/Test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B1ACC3-E026-0A4B-BA57-9595425158E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2372DEE-5B2E-A747-BF4B-677AE3F3572C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="34200" windowHeight="21440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,19 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>Geoffrey Cloud (Med)</t>
-  </si>
-  <si>
-    <t>Daniel Grubman (Med)</t>
-  </si>
-  <si>
-    <t>Katharine Martin (Med)</t>
-  </si>
-  <si>
-    <t>Carolyn Wilson (Med)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>Heidi Dong (ophthal)</t>
   </si>
@@ -70,14 +58,59 @@
     <t>Harmehar Kohli (Med)</t>
   </si>
   <si>
-    <t>OSRs</t>
+    <t>3/9-3/22</t>
+  </si>
+  <si>
+    <t>Availability</t>
+  </si>
+  <si>
+    <t>Amion ID</t>
+  </si>
+  <si>
+    <t>3/9-4/5</t>
+  </si>
+  <si>
+    <t>3/11-3/24</t>
+  </si>
+  <si>
+    <t>3/23-4/5</t>
+  </si>
+  <si>
+    <t>3/25-4/5</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>GN</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>EJ</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>AJ</t>
+  </si>
+  <si>
+    <t>SMe</t>
+  </si>
+  <si>
+    <t>HK</t>
+  </si>
+  <si>
+    <t>OSR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -97,19 +130,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -124,10 +159,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -346,90 +382,136 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="1" t="s">
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="1" t="s">
+      <c r="B6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="1" t="s">
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="1" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="1" t="s">
+      <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="1" t="s">
+      <c r="B10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="1" t="s">
+      <c r="B11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="1" t="s">
-        <v>14</v>
+      <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>